<commit_message>
Add training for level 1, 2 and 3 with 3 sheep
</commit_message>
<xml_diff>
--- a/Mesure.xlsx
+++ b/Mesure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ENSIM\5A\DRL\Git\DeepRenforcementLearning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D448E81-BB16-4E87-820D-EEF81612F4DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA3D3E0-42C0-4D7C-B95E-A609FE3A1EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0806FB1C-282D-4709-952F-DE4506AD4B4F}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="269">
   <si>
     <t>Niveau 1</t>
   </si>
@@ -483,13 +483,658 @@
   </si>
   <si>
     <t>372.5 steps</t>
+  </si>
+  <si>
+    <t>python test.py -t lazy -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t tipsy -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t ruleBase -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python train.py -a ppo -s 3</t>
+  </si>
+  <si>
+    <t>python train.py -a td3 -s 3</t>
+  </si>
+  <si>
+    <t>python train.py -a dqn -s 3</t>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst0_sleepy.zip -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst0_sleepy.zip -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst0_sleepy_best.pth -s 3 -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t lazy -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t tipsy -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t ruleBase -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst0_sleepy.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst0_sleepy.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst0_sleepy_best.pth -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python train.py -a ppo -s 3 --active_sheep -c models/ppo_sheep3_obst0_sleepy.zip -cl</t>
+  </si>
+  <si>
+    <t>python train.py -a td3 -s 3 --active_sheep -c models/td3_sheep3_obst0_sleepy.zip -cl</t>
+  </si>
+  <si>
+    <t>python train.py -a dqn -s 3 --active_sheep -c models/dqn_sheep3_obst0_sleepy_best.pth -cl</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>dqn_sheep3_obst0_active_best.pth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>dqn_sheep3_obst0_curriculum_best.pth</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>td3_sheep3_obst0_active.zip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>td3_sheep3_obst0_curriculum.zip</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ppo_sheep3_obst0_active.zip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ppo_sheep3_obst0_curriculum.zip</t>
+    </r>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst0_curriculum.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst0_curriculum.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst0_curriculum_best.pth -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python train.py -a ppo -s 3 --active_sheep</t>
+  </si>
+  <si>
+    <t>python train.py -a td3 -s 3 --active_sheep</t>
+  </si>
+  <si>
+    <t>python train.py -a dqn -s 3 --active_sheep</t>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst0_active.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst0_active.zip -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst0_active_best.pth -s 3 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t lazy -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t tipsy -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t ruleBase -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst0_active.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst0_active.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst0_active_best.pth -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python train.py -a ppo -s 3 -r 0.2 --active_sheep -c models/ppo_sheep3_obst0_active.zip -cl</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ppo_sheep3_obst2_active.zip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ppo_sheep3_obst2_curriculum.zip</t>
+    </r>
+  </si>
+  <si>
+    <t>python train.py -a td3 -s 3 -r 0.2 --active_sheep -c models/td3_sheep3_obst0_active.zip -cl</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>td3_sheep3_obst2_active.zip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>td3_sheep3_obst2_curriculum.zip</t>
+    </r>
+  </si>
+  <si>
+    <t>python train.py -a dqn -s 3 -r 0.2 --active_sheep -c models/dqn_sheep3_obst0_active_best.pth -cl</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">⚠️ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Renommez</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>dqn_sheep3_obst2_active_best.pth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> en 👉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>dqn_sheep3_obst2_curriculum_best.pth</t>
+    </r>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst2_curriculum.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst2_curriculum.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst2_curriculum_best.pth -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python train.py -a ppo -s 3 -r 0.2 --active_sheep</t>
+  </si>
+  <si>
+    <t>python train.py -a td3 -s 3 -r 0.2 --active_sheep</t>
+  </si>
+  <si>
+    <t>python train.py -a dqn -s 3 -r 0.2 --active_sheep</t>
+  </si>
+  <si>
+    <t>python test.py -t PPO -a models/ppo_sheep3_obst2_active.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t TD3 -a models/td3_sheep3_obst2_active.zip -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>python test.py -t DQN -a models/dqn_sheep3_obst2_active_best.pth -s 3 -r 0.2 --active_sheep -n 100</t>
+  </si>
+  <si>
+    <t>10030.70 ± 5042.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 490.0 steps</t>
+  </si>
+  <si>
+    <t>27281.52 ± 7114.11</t>
+  </si>
+  <si>
+    <t>2.0%</t>
+  </si>
+  <si>
+    <t>495.3 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 17500.22 ± 2004.33</t>
+  </si>
+  <si>
+    <t>94.0%</t>
+  </si>
+  <si>
+    <t>243.6 steps</t>
+  </si>
+  <si>
+    <t>2,149 hr</t>
+  </si>
+  <si>
+    <t>1,516 hr</t>
+  </si>
+  <si>
+    <t>490.0 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 20014.07 ± 6243.83</t>
+  </si>
+  <si>
+    <t>16452.85 ± 5441.18</t>
+  </si>
+  <si>
+    <t>494.3 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 4.0%</t>
+  </si>
+  <si>
+    <t>29615.85 ± 6027.87</t>
+  </si>
+  <si>
+    <t>491.7 steps</t>
+  </si>
+  <si>
+    <t>23393.95 ± 6803.64</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3.0%</t>
+  </si>
+  <si>
+    <t>490.3 steps</t>
+  </si>
+  <si>
+    <t>14205.70 ± 1787.09</t>
+  </si>
+  <si>
+    <t>91.0%</t>
+  </si>
+  <si>
+    <t>217.7 steps</t>
+  </si>
+  <si>
+    <t>23309.69 ± 5972.60</t>
+  </si>
+  <si>
+    <t>26847.31 ± 6231.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 493.8 steps</t>
+  </si>
+  <si>
+    <t>1,046 hr</t>
+  </si>
+  <si>
+    <t>50,61 min</t>
+  </si>
+  <si>
+    <t>28137.94 ± 6709.33</t>
+  </si>
+  <si>
+    <t>3.0%</t>
+  </si>
+  <si>
+    <t>488.3 steps</t>
+  </si>
+  <si>
+    <t>34576.64 ± 7329.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 489.9 steps</t>
+  </si>
+  <si>
+    <t>2,147 hr</t>
+  </si>
+  <si>
+    <t>1,618 hr</t>
+  </si>
+  <si>
+    <t>23283.04 ± 6341.53</t>
+  </si>
+  <si>
+    <t>485.2 steps</t>
+  </si>
+  <si>
+    <t>28781.06 ± 5919.75</t>
+  </si>
+  <si>
+    <t>5.0%</t>
+  </si>
+  <si>
+    <t>482.7 steps</t>
+  </si>
+  <si>
+    <t>27944.23 ± 6426.31</t>
+  </si>
+  <si>
+    <t>495.1 steps</t>
+  </si>
+  <si>
+    <t>26996.21 ± 5707.25</t>
+  </si>
+  <si>
+    <t>0.0%</t>
+  </si>
+  <si>
+    <t>500.0 steps</t>
+  </si>
+  <si>
+    <t>16098.12 ± 2525.83</t>
+  </si>
+  <si>
+    <t>76.0%</t>
+  </si>
+  <si>
+    <t>289.3 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 22110.54 ± 6339.64</t>
+  </si>
+  <si>
+    <t>495.2 steps</t>
+  </si>
+  <si>
+    <t>21028.18 ± 5957.76</t>
+  </si>
+  <si>
+    <t>1.0%</t>
+  </si>
+  <si>
+    <t>495.0 steps</t>
+  </si>
+  <si>
+    <t>1,198 hr</t>
+  </si>
+  <si>
+    <t>48,49 min</t>
+  </si>
+  <si>
+    <t>16320.07 ± 5459.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 487.8 steps</t>
+  </si>
+  <si>
+    <t>32233.59 ± 6898.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 481.5 steps</t>
+  </si>
+  <si>
+    <t>1,992 hr</t>
+  </si>
+  <si>
+    <t>1,566 hr</t>
+  </si>
+  <si>
+    <t>25283.18 ± 6601.89</t>
+  </si>
+  <si>
+    <t>489.1 steps</t>
+  </si>
+  <si>
+    <t>26069.88 ± 6775.21</t>
+  </si>
+  <si>
+    <t>481.4 steps</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -517,6 +1162,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -672,7 +1322,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -692,7 +1342,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -702,11 +1351,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -739,6 +1386,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -760,28 +1411,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1119,7 +1750,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0744EF66-6EF5-4E6D-8377-EBF08112D5D6}">
   <dimension ref="B2:Q11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="71" bestFit="1" customWidth="1"/>
@@ -1128,50 +1759,51 @@
     <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="71" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="2:17">
+      <c r="B2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="K2" s="29" t="s">
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="K2" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-    </row>
-    <row r="3" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+    </row>
+    <row r="3" spans="2:17" ht="15.75" thickBot="1"/>
+    <row r="4" spans="2:17" ht="24.75" thickBot="1">
       <c r="B4" s="1"/>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="26" t="s">
+      <c r="M4" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="28"/>
-    </row>
-    <row r="5" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N4" s="26"/>
+      <c r="O4" s="27"/>
+    </row>
+    <row r="5" spans="2:17" ht="15.75" thickBot="1">
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
         <v>28</v>
@@ -1179,16 +1811,16 @@
       <c r="D5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="38" t="s">
+      <c r="G5" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H5" s="38" t="s">
+      <c r="H5" s="24" t="s">
         <v>73</v>
       </c>
       <c r="K5" s="1"/>
@@ -1196,24 +1828,24 @@
       <c r="M5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="N5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P5" s="38" t="s">
+      <c r="P5" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="Q5" s="38" t="s">
+      <c r="Q5" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17">
       <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="21" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="5" t="s">
@@ -1222,51 +1854,67 @@
       <c r="E6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
       <c r="K6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="4"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="35"/>
-      <c r="Q6" s="35"/>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="8" t="s">
+      <c r="L6" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+    </row>
+    <row r="7" spans="2:17">
+      <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="K7" s="8" t="s">
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="K7" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="L7" s="1"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="35"/>
-      <c r="Q7" s="35"/>
-    </row>
-    <row r="8" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="8" t="s">
+      <c r="L7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="O7" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="23"/>
+    </row>
+    <row r="8" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B8" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
@@ -1275,41 +1923,49 @@
       <c r="D8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="K8" s="8" t="s">
+      <c r="G8" s="23"/>
+      <c r="H8" s="23"/>
+      <c r="K8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="L8" s="1"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="35"/>
-      <c r="Q8" s="35"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L8" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="O8" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="23"/>
+    </row>
+    <row r="9" spans="2:17">
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="G9" s="3" t="s">
         <v>77</v>
       </c>
       <c r="H9" s="3" t="s">
@@ -1318,76 +1974,104 @@
       <c r="K9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="34"/>
-      <c r="Q9" s="3"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
+      <c r="L9" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="O9" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="36" t="s">
+      <c r="G10" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="K10" s="8" t="s">
+      <c r="K10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="L10" s="1"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="8"/>
-    </row>
-    <row r="11" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="14" t="s">
+      <c r="L10" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M10" s="8"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="22" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="37" t="s">
+      <c r="G11" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="H11" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="K11" s="14" t="s">
+      <c r="K11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="L11" s="15"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="37"/>
-      <c r="Q11" s="14"/>
+      <c r="L11" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="O11" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="P11" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q11" s="11" t="s">
+        <v>157</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1402,8 +2086,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8F0C723-653A-4E8B-BD64-04ABCDEBBBC0}">
-  <dimension ref="B2:Q32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:R32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="90.7109375" bestFit="1" customWidth="1"/>
@@ -1413,59 +2097,60 @@
     <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="84" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="88.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="43" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="82.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="85.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="2:17">
+      <c r="B2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="K2" s="29" t="s">
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="K2" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-    </row>
-    <row r="3" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:17" ht="24" x14ac:dyDescent="0.4">
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+    </row>
+    <row r="3" spans="2:17" ht="15.75" thickBot="1"/>
+    <row r="4" spans="2:17" ht="24">
       <c r="B4" s="1"/>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
-      <c r="H4" s="19" t="s">
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
+      <c r="H4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="18"/>
+      <c r="I4" s="15"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="26" t="s">
+      <c r="M4" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="28"/>
-      <c r="Q4" s="21" t="s">
+      <c r="N4" s="26"/>
+      <c r="O4" s="27"/>
+      <c r="Q4" s="18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="15.75" thickBot="1">
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -1473,14 +2158,14 @@
       <c r="D5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="33"/>
-      <c r="H5" s="20"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="17"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
         <v>8</v>
@@ -1488,16 +2173,16 @@
       <c r="M5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="N5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+    </row>
+    <row r="6" spans="2:17">
       <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
@@ -1510,51 +2195,61 @@
       <c r="E6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="39"/>
-      <c r="H6" s="20"/>
+      <c r="H6" s="17"/>
       <c r="K6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="4"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="39"/>
-      <c r="Q6" s="39"/>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="8" t="s">
+      <c r="L6" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="7" spans="2:17">
+      <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="20"/>
-      <c r="K7" s="8" t="s">
+      <c r="H7" s="17"/>
+      <c r="K7" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="L7" s="1"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-    </row>
-    <row r="8" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="8" t="s">
+      <c r="L7" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="O7" s="20" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B8" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -1563,149 +2258,178 @@
       <c r="D8" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="20"/>
-      <c r="K8" s="8" t="s">
+      <c r="H8" s="17"/>
+      <c r="K8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="L8" s="1"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="39"/>
-      <c r="Q8" s="39"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L8" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="O8" s="13" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="9" spans="2:17">
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="33"/>
-      <c r="H9" s="20"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="17"/>
       <c r="K9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="40"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
+      <c r="L9" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="O9" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+    </row>
+    <row r="10" spans="2:17">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="G10" s="33"/>
-      <c r="H10" s="20"/>
-      <c r="K10" s="8" t="s">
+      <c r="G10" s="1"/>
+      <c r="H10" s="17"/>
+      <c r="K10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="1"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="40"/>
-    </row>
-    <row r="11" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="14" t="s">
+      <c r="L10" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="M10" s="8"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+    </row>
+    <row r="11" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="12" t="s">
         <v>69</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="G11" s="33"/>
-      <c r="H11" s="20"/>
-      <c r="K11" s="14" t="s">
+      <c r="G11" s="1"/>
+      <c r="H11" s="17"/>
+      <c r="K11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L11" s="15"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="33"/>
-      <c r="Q11" s="40"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L11" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="O11" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+    </row>
+    <row r="12" spans="2:17">
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="H12" s="20"/>
-      <c r="Q12" s="20"/>
-    </row>
-    <row r="13" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="17"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="Q12" s="17"/>
+    </row>
+    <row r="13" spans="2:17" ht="15.75" thickBot="1">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="H13" s="20"/>
-      <c r="Q13" s="20"/>
-    </row>
-    <row r="14" spans="2:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H13" s="17"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="Q13" s="17"/>
+    </row>
+    <row r="14" spans="2:17" ht="24.75" thickBot="1">
       <c r="B14" s="1"/>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
-      <c r="H14" s="21" t="s">
+      <c r="E14" s="26"/>
+      <c r="F14" s="27"/>
+      <c r="H14" s="18" t="s">
         <v>12</v>
       </c>
       <c r="K14" s="1"/>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M14" s="30" t="s">
+      <c r="M14" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="N14" s="31"/>
-      <c r="O14" s="32"/>
-      <c r="Q14" s="21" t="s">
+      <c r="N14" s="30"/>
+      <c r="O14" s="31"/>
+      <c r="Q14" s="18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:17" ht="15.75" thickBot="1">
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
         <v>10</v>
@@ -1713,16 +2437,16 @@
       <c r="D15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="38" t="s">
+      <c r="G15" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="38" t="s">
+      <c r="H15" s="24" t="s">
         <v>73</v>
       </c>
       <c r="K15" s="1"/>
@@ -1732,96 +2456,96 @@
       <c r="M15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N15" s="15" t="s">
+      <c r="N15" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O15" s="16" t="s">
+      <c r="O15" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P15" s="38" t="s">
+      <c r="P15" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="Q15" s="38" t="s">
+      <c r="Q15" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:17">
       <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
       <c r="K16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="5"/>
       <c r="N16" s="6"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="8" t="s">
+      <c r="O16" s="19"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+    </row>
+    <row r="17" spans="2:18">
+      <c r="B17" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C17" s="1"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="K17" s="8" t="s">
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="K17" s="7" t="s">
         <v>2</v>
       </c>
       <c r="L17" s="1"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="35"/>
-      <c r="Q17" s="35"/>
-    </row>
-    <row r="18" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="8" t="s">
+      <c r="M17" s="8"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+    </row>
+    <row r="18" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B18" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="K18" s="8" t="s">
+      <c r="E18" s="10"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="K18" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="12"/>
+      <c r="N18" s="10"/>
       <c r="O18" s="13"/>
-      <c r="P18" s="35"/>
-      <c r="Q18" s="35"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
+    </row>
+    <row r="19" spans="2:18">
       <c r="B19" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="3" t="s">
         <v>93</v>
       </c>
       <c r="H19" s="3" t="s">
@@ -1830,110 +2554,153 @@
       <c r="K19" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L19" s="4"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="34"/>
-      <c r="Q19" s="3"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
+      <c r="L19" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O19" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q19" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="R19" s="32" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18">
+      <c r="B20" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="8" t="s">
+      <c r="D20" s="8"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K20" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="1"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="8"/>
-    </row>
-    <row r="21" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="14" t="s">
+      <c r="L20" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="M20" s="8"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="20"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="R20" s="32" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B21" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="12" t="s">
         <v>84</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="G21" s="37" t="s">
+      <c r="G21" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="K21" s="14" t="s">
+      <c r="K21" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="37"/>
-      <c r="Q21" s="14"/>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L21" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="N21" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="P21" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q21" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="R21" s="32" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="H22" s="20"/>
-      <c r="Q22" s="20"/>
-    </row>
-    <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="17"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="Q22" s="17"/>
+    </row>
+    <row r="23" spans="2:18" ht="15.75" thickBot="1">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-      <c r="H23" s="20"/>
-      <c r="Q23" s="20"/>
-    </row>
-    <row r="24" spans="2:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H23" s="17"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="Q23" s="17"/>
+    </row>
+    <row r="24" spans="2:18" ht="24.75" thickBot="1">
       <c r="B24" s="1"/>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="28"/>
-      <c r="H24" s="21" t="s">
+      <c r="E24" s="26"/>
+      <c r="F24" s="27"/>
+      <c r="H24" s="18" t="s">
         <v>13</v>
       </c>
       <c r="K24" s="1"/>
-      <c r="L24" s="17" t="s">
+      <c r="L24" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M24" s="26" t="s">
+      <c r="M24" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="N24" s="27"/>
-      <c r="O24" s="28"/>
-      <c r="Q24" s="21" t="s">
+      <c r="N24" s="26"/>
+      <c r="O24" s="27"/>
+      <c r="Q24" s="18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:18" ht="15.75" thickBot="1">
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
         <v>81</v>
@@ -1941,16 +2708,16 @@
       <c r="D25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="F25" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G25" s="38" t="s">
+      <c r="G25" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H25" s="38" t="s">
+      <c r="H25" s="24" t="s">
         <v>73</v>
       </c>
       <c r="K25" s="1"/>
@@ -1960,96 +2727,96 @@
       <c r="M25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N25" s="15" t="s">
+      <c r="N25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O25" s="16" t="s">
+      <c r="O25" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P25" s="38" t="s">
+      <c r="P25" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="Q25" s="38" t="s">
+      <c r="Q25" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:18">
       <c r="B26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="35"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
       <c r="K26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="5"/>
       <c r="N26" s="6"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="35"/>
-      <c r="Q26" s="35"/>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B27" s="8" t="s">
+      <c r="O26" s="19"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="23"/>
+    </row>
+    <row r="27" spans="2:18">
+      <c r="B27" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C27" s="1"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="K27" s="8" t="s">
+      <c r="D27" s="8"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="K27" s="7" t="s">
         <v>2</v>
       </c>
       <c r="L27" s="1"/>
-      <c r="M27" s="9"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="11"/>
-      <c r="P27" s="35"/>
-      <c r="Q27" s="35"/>
-    </row>
-    <row r="28" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="8" t="s">
+      <c r="M27" s="8"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="20"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="23"/>
+    </row>
+    <row r="28" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B28" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="K28" s="8" t="s">
+      <c r="E28" s="10"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="K28" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="2"/>
-      <c r="N28" s="12"/>
+      <c r="N28" s="10"/>
       <c r="O28" s="13"/>
-      <c r="P28" s="35"/>
-      <c r="Q28" s="35"/>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+    </row>
+    <row r="29" spans="2:18">
       <c r="B29" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="G29" s="34" t="s">
+      <c r="G29" s="3" t="s">
         <v>100</v>
       </c>
       <c r="H29" s="3" t="s">
@@ -2058,70 +2825,101 @@
       <c r="K29" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L29" s="4"/>
-      <c r="M29" s="9"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="11"/>
-      <c r="P29" s="34"/>
-      <c r="Q29" s="3"/>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="8" t="s">
+      <c r="L29" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="M29" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="N29" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O29" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q29" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="R29" s="32"/>
+    </row>
+    <row r="30" spans="2:18">
+      <c r="B30" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="8" t="s">
+      <c r="D30" s="8"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="K30" s="8" t="s">
+      <c r="K30" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L30" s="1"/>
-      <c r="M30" s="9"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="11"/>
-      <c r="P30" s="36"/>
-      <c r="Q30" s="8"/>
-    </row>
-    <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="14" t="s">
+      <c r="L30" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="M30" s="8"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="20"/>
+      <c r="P30" s="7"/>
+      <c r="Q30" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="R30" s="32"/>
+    </row>
+    <row r="31" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="12" t="s">
         <v>92</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F31" s="16" t="s">
+      <c r="F31" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="G31" s="37" t="s">
+      <c r="G31" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="H31" s="14" t="s">
+      <c r="H31" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="K31" s="14" t="s">
+      <c r="K31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="12"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="37"/>
-      <c r="Q31" s="14"/>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L31" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="N31" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="O31" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="P31" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q31" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="R31" s="32"/>
+    </row>
+    <row r="32" spans="2:18">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -2138,13 +2936,14 @@
     <mergeCell ref="D4:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD226A34-13FF-4F4D-A688-C597425C2EF8}">
-  <dimension ref="B2:Q32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:R32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="95.7109375" bestFit="1" customWidth="1"/>
@@ -2154,58 +2953,58 @@
     <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="88.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="93.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="43" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="86.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="85.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="29" t="s">
+    <row r="2" spans="2:17">
+      <c r="B2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="K2" s="29" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-    </row>
-    <row r="3" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:17" ht="24" x14ac:dyDescent="0.4">
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="K2" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+    </row>
+    <row r="3" spans="2:17" ht="15.75" thickBot="1"/>
+    <row r="4" spans="2:17" ht="24">
       <c r="B4" s="1"/>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="28"/>
-      <c r="H4" s="21" t="s">
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
+      <c r="H4" s="18" t="s">
         <v>17</v>
       </c>
       <c r="K4" s="1"/>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="26" t="s">
+      <c r="M4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="28"/>
-      <c r="Q4" s="21" t="s">
+      <c r="N4" s="26"/>
+      <c r="O4" s="27"/>
+      <c r="Q4" s="18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="15.75" thickBot="1">
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -2213,14 +3012,14 @@
       <c r="D5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="F5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="33"/>
-      <c r="H5" s="20"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="17"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
         <v>8</v>
@@ -2228,16 +3027,16 @@
       <c r="M5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="N5" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O5" s="16" t="s">
+      <c r="O5" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="20"/>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P5" s="1"/>
+      <c r="Q5" s="17"/>
+    </row>
+    <row r="6" spans="2:17">
       <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
@@ -2250,51 +3049,63 @@
       <c r="E6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="G6" s="39"/>
-      <c r="H6" s="20"/>
+      <c r="H6" s="17"/>
       <c r="K6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L6" s="4"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="39"/>
-      <c r="Q6" s="20"/>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="8" t="s">
+      <c r="L6" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q6" s="17"/>
+    </row>
+    <row r="7" spans="2:17">
+      <c r="B7" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="20"/>
-      <c r="K7" s="8" t="s">
+      <c r="H7" s="17"/>
+      <c r="K7" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="L7" s="1"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="20"/>
-    </row>
-    <row r="8" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="8" t="s">
+      <c r="L7" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="O7" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="Q7" s="17"/>
+    </row>
+    <row r="8" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B8" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -2303,143 +3114,173 @@
       <c r="D8" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="20"/>
-      <c r="K8" s="8" t="s">
+      <c r="H8" s="17"/>
+      <c r="K8" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="L8" s="1"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="39"/>
-      <c r="Q8" s="20"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L8" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="N8" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="O8" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="Q8" s="17"/>
+    </row>
+    <row r="9" spans="2:17">
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="G9" s="33"/>
-      <c r="H9" s="20"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="17"/>
       <c r="K9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="20"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="8" t="s">
+      <c r="L9" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="O9" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="17"/>
+    </row>
+    <row r="10" spans="2:17">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="20"/>
-      <c r="K10" s="8" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="17"/>
+      <c r="K10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L10" s="1"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="20"/>
-    </row>
-    <row r="11" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="14" t="s">
+      <c r="L10" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="M10" s="8"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="20"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="17"/>
+    </row>
+    <row r="11" spans="2:17" ht="15.75" thickBot="1">
+      <c r="B11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="12" t="s">
         <v>123</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="G11" s="33"/>
-      <c r="H11" s="20"/>
-      <c r="K11" s="14" t="s">
+      <c r="G11" s="1"/>
+      <c r="H11" s="17"/>
+      <c r="K11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L11" s="15"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="33"/>
-      <c r="Q11" s="20"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L11" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>255</v>
+      </c>
+      <c r="O11" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="17"/>
+    </row>
+    <row r="12" spans="2:17">
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="H12" s="20"/>
-      <c r="Q12" s="20"/>
-    </row>
-    <row r="13" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="17"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="Q12" s="17"/>
+    </row>
+    <row r="13" spans="2:17" ht="15.75" thickBot="1">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="H13" s="20"/>
-      <c r="Q13" s="20"/>
-    </row>
-    <row r="14" spans="2:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H13" s="17"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="Q13" s="17"/>
+    </row>
+    <row r="14" spans="2:17" ht="24.75" thickBot="1">
       <c r="B14" s="1"/>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
-      <c r="H14" s="21" t="s">
+      <c r="E14" s="26"/>
+      <c r="F14" s="27"/>
+      <c r="H14" s="18" t="s">
         <v>12</v>
       </c>
       <c r="K14" s="1"/>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M14" s="26" t="s">
+      <c r="M14" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="N14" s="27"/>
-      <c r="O14" s="28"/>
-      <c r="Q14" s="21" t="s">
+      <c r="N14" s="26"/>
+      <c r="O14" s="27"/>
+      <c r="Q14" s="18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:17" ht="15.75" thickBot="1">
       <c r="B15" s="1"/>
       <c r="C15" s="1" t="s">
         <v>10</v>
@@ -2447,16 +3288,16 @@
       <c r="D15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="38" t="s">
+      <c r="G15" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="38" t="s">
+      <c r="H15" s="24" t="s">
         <v>73</v>
       </c>
       <c r="K15" s="1"/>
@@ -2466,96 +3307,96 @@
       <c r="M15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N15" s="15" t="s">
+      <c r="N15" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O15" s="16" t="s">
+      <c r="O15" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P15" s="38" t="s">
+      <c r="P15" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="Q15" s="38" t="s">
+      <c r="Q15" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:17">
       <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
       <c r="E16" s="6"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
       <c r="K16" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="5"/>
       <c r="N16" s="6"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="8" t="s">
+      <c r="O16" s="19"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+    </row>
+    <row r="17" spans="2:18">
+      <c r="B17" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C17" s="1"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="35"/>
-      <c r="K17" s="8" t="s">
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="K17" s="7" t="s">
         <v>2</v>
       </c>
       <c r="L17" s="1"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="35"/>
-      <c r="Q17" s="35"/>
-    </row>
-    <row r="18" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="8" t="s">
+      <c r="M17" s="8"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+    </row>
+    <row r="18" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B18" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="K18" s="8" t="s">
+      <c r="E18" s="10"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="K18" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="12"/>
+      <c r="N18" s="10"/>
       <c r="O18" s="13"/>
-      <c r="P18" s="35"/>
-      <c r="Q18" s="35"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
+    </row>
+    <row r="19" spans="2:18">
       <c r="B19" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="E19" s="40" t="s">
+      <c r="E19" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="20" t="s">
         <v>142</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="3" t="s">
         <v>138</v>
       </c>
       <c r="H19" s="3" t="s">
@@ -2564,109 +3405,152 @@
       <c r="K19" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L19" s="4"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="34"/>
-      <c r="Q19" s="3"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="8" t="s">
+      <c r="L19" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O19" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="P19" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q19" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="R19" s="32" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="20" spans="2:18">
+      <c r="B20" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="10"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="8" t="s">
+      <c r="D20" s="8"/>
+      <c r="E20" s="9"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K20" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="1"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="8"/>
-    </row>
-    <row r="21" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="14" t="s">
+      <c r="L20" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="M20" s="8"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="20"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="R20" s="32" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B21" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="12" t="s">
         <v>131</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="16" t="s">
+      <c r="F21" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="G21" s="37" t="s">
+      <c r="G21" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="H21" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="K21" s="14" t="s">
+      <c r="K21" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="12"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="37"/>
-      <c r="Q21" s="14"/>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L21" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="N21" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="P21" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q21" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="R21" s="32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="H22" s="20"/>
-      <c r="Q22" s="20"/>
-    </row>
-    <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="17"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="Q22" s="17"/>
+    </row>
+    <row r="23" spans="2:18" ht="15.75" thickBot="1">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-      <c r="H23" s="20"/>
-      <c r="Q23" s="20"/>
-    </row>
-    <row r="24" spans="2:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="H23" s="17"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="Q23" s="17"/>
+    </row>
+    <row r="24" spans="2:18" ht="24.75" thickBot="1">
       <c r="B24" s="1"/>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="28"/>
-      <c r="H24" s="21" t="s">
+      <c r="E24" s="26"/>
+      <c r="F24" s="27"/>
+      <c r="H24" s="18" t="s">
         <v>13</v>
       </c>
       <c r="K24" s="1"/>
-      <c r="L24" s="17" t="s">
+      <c r="L24" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="M24" s="26" t="s">
+      <c r="M24" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="N24" s="27"/>
-      <c r="O24" s="28"/>
-      <c r="Q24" s="21" t="s">
+      <c r="N24" s="26"/>
+      <c r="O24" s="27"/>
+      <c r="Q24" s="18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:18" ht="15.75" thickBot="1">
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
         <v>81</v>
@@ -2674,16 +3558,16 @@
       <c r="D25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="16" t="s">
+      <c r="F25" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G25" s="38" t="s">
+      <c r="G25" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="H25" s="38" t="s">
+      <c r="H25" s="24" t="s">
         <v>73</v>
       </c>
       <c r="K25" s="1"/>
@@ -2693,96 +3577,96 @@
       <c r="M25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N25" s="15" t="s">
+      <c r="N25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="O25" s="16" t="s">
+      <c r="O25" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P25" s="38" t="s">
+      <c r="P25" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="Q25" s="38" t="s">
+      <c r="Q25" s="24" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:18">
       <c r="B26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="35"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
       <c r="K26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="5"/>
       <c r="N26" s="6"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="35"/>
-      <c r="Q26" s="35"/>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B27" s="8" t="s">
+      <c r="O26" s="19"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="23"/>
+    </row>
+    <row r="27" spans="2:18">
+      <c r="B27" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C27" s="1"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="K27" s="8" t="s">
+      <c r="D27" s="8"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="K27" s="7" t="s">
         <v>2</v>
       </c>
       <c r="L27" s="1"/>
-      <c r="M27" s="9"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="11"/>
-      <c r="P27" s="35"/>
-      <c r="Q27" s="35"/>
-    </row>
-    <row r="28" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="8" t="s">
+      <c r="M27" s="8"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="20"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="23"/>
+    </row>
+    <row r="28" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B28" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="K28" s="8" t="s">
+      <c r="E28" s="10"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="K28" s="7" t="s">
         <v>3</v>
       </c>
       <c r="L28" s="1"/>
       <c r="M28" s="2"/>
-      <c r="N28" s="12"/>
+      <c r="N28" s="10"/>
       <c r="O28" s="13"/>
-      <c r="P28" s="35"/>
-      <c r="Q28" s="35"/>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+    </row>
+    <row r="29" spans="2:18">
       <c r="B29" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="G29" s="34" t="s">
+      <c r="G29" s="3" t="s">
         <v>145</v>
       </c>
       <c r="H29" s="3" t="s">
@@ -2791,70 +3675,98 @@
       <c r="K29" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="L29" s="4"/>
-      <c r="M29" s="9"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="11"/>
-      <c r="P29" s="34"/>
-      <c r="Q29" s="3"/>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="8" t="s">
+      <c r="L29" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="M29" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="N29" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="O29" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q29" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="30" spans="2:18">
+      <c r="B30" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="D30" s="9"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="8" t="s">
+      <c r="D30" s="8"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="20"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="K30" s="8" t="s">
+      <c r="K30" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="L30" s="1"/>
-      <c r="M30" s="9"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="11"/>
-      <c r="P30" s="36"/>
-      <c r="Q30" s="8"/>
-    </row>
-    <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="14" t="s">
+      <c r="L30" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="M30" s="8"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="20"/>
+      <c r="P30" s="7"/>
+      <c r="Q30" s="7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="31" spans="2:18" ht="15.75" thickBot="1">
+      <c r="B31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="12" t="s">
         <v>137</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E31" s="12" t="s">
+      <c r="E31" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="F31" s="16" t="s">
+      <c r="F31" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G31" s="37" t="s">
+      <c r="G31" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="H31" s="14" t="s">
+      <c r="H31" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="K31" s="14" t="s">
+      <c r="K31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="12"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="37"/>
-      <c r="Q31" s="14"/>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="L31" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="N31" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="O31" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="P31" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q31" s="11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="32" spans="2:18">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>

</xml_diff>

<commit_message>
Update README.md for clarity and feature highlights; add new video presentation
</commit_message>
<xml_diff>
--- a/Mesure.xlsx
+++ b/Mesure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\ENSIM\5A\DRL\Git\DeepRenforcementLearning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4110B265-8891-48BC-B9D4-D78753BEC455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2153FF60-032E-498E-8CDC-490B4444CD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0806FB1C-282D-4709-952F-DE4506AD4B4F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0806FB1C-282D-4709-952F-DE4506AD4B4F}"/>
   </bookViews>
   <sheets>
     <sheet name="Level 1" sheetId="1" r:id="rId1"/>

</xml_diff>